<commit_message>
test: stabilize phase 1 against production site
- TC-REK-001: heading "daftar rekening" ditulis huruf kecil di DOM
  (kapital dari CSS), cocokkan tanpa membedakan huruf besar/kecil
- TC-PAY-010: picu blur sebelum cek filter nama, karena
  validateNameInput() berjalan saat onchange
- TC-PAY-012..014: lepas tag @known-bug, temuan F-14 sudah diperbaiki
  di situs (next_step() kini memvalidasi seluruh field)
- Perbarui test plan, README, dan PANDUAN sesuai hasil verifikasi

npm test hijau 2x berturut-turut (39/39); test:known-bug: 3 gagal
sesuai temuan F-01, F-12, F-15.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Test_Plan_Cypress_BAZNAS.xlsx
+++ b/docs/Test_Plan_Cypress_BAZNAS.xlsx
@@ -7814,7 +7814,7 @@
       </c>
       <c r="J59" s="18" t="inlineStr">
         <is>
-          <t>@regression @known-bug</t>
+          <t>@regression</t>
         </is>
       </c>
       <c r="K59" s="18" t="inlineStr">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>@known-bug – temuan F-14</t>
+          <t>Temuan F-14 sudah diperbaiki di situs (diverifikasi 27 Okt 2026); tag @known-bug dilepas</t>
         </is>
       </c>
       <c r="O59" s="19" t="inlineStr">
@@ -7897,7 +7897,7 @@
       </c>
       <c r="J60" s="18" t="inlineStr">
         <is>
-          <t>@regression @known-bug</t>
+          <t>@regression</t>
         </is>
       </c>
       <c r="K60" s="18" t="inlineStr">
@@ -7917,7 +7917,7 @@
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>@known-bug – temuan F-14</t>
+          <t>Temuan F-14 sudah diperbaiki di situs (diverifikasi 27 Okt 2026); tag @known-bug dilepas</t>
         </is>
       </c>
       <c r="O60" s="19" t="inlineStr">
@@ -7980,7 +7980,7 @@
       </c>
       <c r="J61" s="18" t="inlineStr">
         <is>
-          <t>@regression @known-bug</t>
+          <t>@regression</t>
         </is>
       </c>
       <c r="K61" s="18" t="inlineStr">
@@ -8000,7 +8000,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>@known-bug – temuan F-14</t>
+          <t>Temuan F-14 sudah diperbaiki di situs (diverifikasi 27 Okt 2026); tag @known-bug dilepas</t>
         </is>
       </c>
       <c r="O61" s="19" t="inlineStr">
@@ -12883,12 +12883,12 @@
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>Terkonfirmasi untuk field kosong (request ke server diblokir saat eksplorasi)</t>
+          <t>Sudah diperbaiki (diverifikasi ulang 27 Okt 2026: next_step() menjalankan validasi seluruh field)</t>
         </is>
       </c>
       <c r="I15" s="19" t="inlineStr">
         <is>
-          <t>TC-PAY-012..014 (@known-bug)</t>
+          <t>TC-PAY-012..014 (lulus, tag @known-bug dilepas)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: add phase 2 batch A (forms & calculator)
28 test case P2/P3:
- Kalkulator: nominal besar, input tidak valid, field kosong, field hasil
  read-only, tombol Sedekah, dropdown jenis, perusahaan, perdagangan, emas
- Form bayar zakat: sub-jenis infak/sedekah, nominal saat ganti jenis dana,
  opsi hari fidyah, nominal nol, pernyataan muzaki, logo metode, tab Kalkulator
- Jemput zakat: kelengkapan form, opsi, captcha, HP berisi huruf, tanggal lampau
- Spec baru konfirmasi-zis dan newsletter (request Mailchimp di-stub)

Known-bug baru: TC-CALC-010 (F-19), TC-PAY-006 (F-05), TC-JMP-003 (F-20),
TC-JMP-008 (F-09), TC-KONF-001 (F-02). Temuan baru F-17..F-20 dicatat di
test plan.

Spec yang diubah hijau 2x berturut-turut (46/46).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Test_Plan_Cypress_BAZNAS.xlsx
+++ b/docs/Test_Plan_Cypress_BAZNAS.xlsx
@@ -5969,7 +5969,7 @@
       </c>
       <c r="J36" s="18" t="inlineStr">
         <is>
-          <t>@regression</t>
+          <t>@regression @known-bug</t>
         </is>
       </c>
       <c r="K36" s="18" t="inlineStr">
@@ -5987,7 +5987,11 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="N36" s="19" t="n"/>
+      <c r="N36" s="19" t="inlineStr">
+        <is>
+          <t>@known-bug – temuan F-19 (koma diterima oleh mask input)</t>
+        </is>
+      </c>
       <c r="O36" s="19" t="inlineStr">
         <is>
           <t>cypress/e2e/kalkulator-zakat.cy.ts</t>
@@ -6627,7 +6631,7 @@
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>Rumus dikonfirmasi ke tim bisnis</t>
+          <t>Rumus dari script halaman: Jasa = 2,5% x pendapatan sebelum pajak; Dagang/Industri = 2,5% x (aktiva lancar - pasiva lancar); wajib jika &gt;= nisab per tahun. Perlu konfirmasi tim bisnis. Lihat temuan F-17</t>
         </is>
       </c>
       <c r="O44" s="19" t="inlineStr">
@@ -6708,7 +6712,11 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="N45" s="19" t="n"/>
+      <c r="N45" s="19" t="inlineStr">
+        <is>
+          <t>Rumus dari script halaman: 2,5% x (aset lancar + laba), wajib jika &gt;= nisab per tahun. Perlu konfirmasi tim bisnis. Lihat temuan F-17</t>
+        </is>
+      </c>
       <c r="O45" s="19" t="inlineStr">
         <is>
           <t>cypress/e2e/kalkulator-zakat.cy.ts</t>
@@ -6788,7 +6796,11 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="N46" s="19" t="n"/>
+      <c r="N46" s="19" t="inlineStr">
+        <is>
+          <t>Rumus dari script halaman: 2,5% x (gram x harga per gram), dibulatkan ke atas; wajib jika &gt;= 85 gram</t>
+        </is>
+      </c>
       <c r="O46" s="19" t="inlineStr">
         <is>
           <t>cypress/e2e/kalkulator-zakat.cy.ts</t>
@@ -7327,7 +7339,7 @@
       </c>
       <c r="J53" s="18" t="inlineStr">
         <is>
-          <t>@regression</t>
+          <t>@regression @known-bug</t>
         </is>
       </c>
       <c r="K53" s="18" t="inlineStr">
@@ -7347,7 +7359,7 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>Lihat temuan F-05</t>
+          <t>@known-bug – temuan F-05</t>
         </is>
       </c>
       <c r="O53" s="19" t="inlineStr">
@@ -8081,7 +8093,11 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="N62" s="19" t="n"/>
+      <c r="N62" s="19" t="inlineStr">
+        <is>
+          <t>Formulir tetap lanjut dengan nominal 0; batas minimum diterapkan di layar Metode Pembayaran (metode dinonaktifkan, "Minimal pembayaran Rp10.000"). Tidak ada metode yang diklik</t>
+        </is>
+      </c>
       <c r="O62" s="19" t="inlineStr">
         <is>
           <t>cypress/e2e/bayar-zakat.cy.ts</t>
@@ -8480,7 +8496,7 @@
       </c>
       <c r="N67" s="19" t="inlineStr">
         <is>
-          <t>Rumus dikonfirmasi ke tim bisnis</t>
+          <t>Rumus dari script halaman: 2,5% x (emas/perak + tabungan + kendaraan - hutang). Perlu konfirmasi tim bisnis. Lihat temuan F-18</t>
         </is>
       </c>
       <c r="O67" s="19" t="inlineStr">
@@ -8699,7 +8715,7 @@
       </c>
       <c r="J70" s="18" t="inlineStr">
         <is>
-          <t>@regression</t>
+          <t>@regression @known-bug</t>
         </is>
       </c>
       <c r="K70" s="18" t="inlineStr">
@@ -8719,7 +8735,7 @@
       </c>
       <c r="N70" s="19" t="inlineStr">
         <is>
-          <t>Captcha tidak diselesaikan otomatis</t>
+          <t>@known-bug – temuan F-20 (gambar captcha gagal dimuat). Captcha tidak diselesaikan otomatis</t>
         </is>
       </c>
       <c r="O70" s="19" t="inlineStr">
@@ -8963,7 +8979,7 @@
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>Tidak ada atribut pattern pada field HP</t>
+          <t>Huruf ditolak saat diketik (hanyaAngka). Pesan invalid-feedback baru tampil setelah captcha benar; captcha di-stub "false", jadi yang dicek constraint validation</t>
         </is>
       </c>
       <c r="O73" s="19" t="inlineStr">
@@ -9109,7 +9125,7 @@
       </c>
       <c r="J75" s="18" t="inlineStr">
         <is>
-          <t>@regression</t>
+          <t>@regression @known-bug</t>
         </is>
       </c>
       <c r="K75" s="18" t="inlineStr">
@@ -9129,7 +9145,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Lihat temuan F-09</t>
+          <t>@known-bug – temuan F-09</t>
         </is>
       </c>
       <c r="O75" s="19" t="inlineStr">
@@ -9191,7 +9207,7 @@
       </c>
       <c r="J76" s="18" t="inlineStr">
         <is>
-          <t>@regression</t>
+          <t>@regression @known-bug</t>
         </is>
       </c>
       <c r="K76" s="18" t="inlineStr">
@@ -9211,7 +9227,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Lihat temuan F-02 (typo heading)</t>
+          <t>@known-bug – temuan F-02 (typo heading)</t>
         </is>
       </c>
       <c r="O76" s="19" t="inlineStr">
@@ -12214,7 +12230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="10" min="1" max="1"/>
@@ -12362,7 +12378,11 @@
           <t>Terkonfirmasi</t>
         </is>
       </c>
-      <c r="I3" s="19" t="n"/>
+      <c r="I3" s="19" t="inlineStr">
+        <is>
+          <t>TC-KONF-001 (@known-bug)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="23.85" customHeight="1" s="11">
       <c r="A4" s="18" t="inlineStr">
@@ -12488,10 +12508,14 @@
       </c>
       <c r="H6" s="19" t="inlineStr">
         <is>
-          <t>Terkonfirmasi (perlu cek ulang apakah field kembali editable)</t>
-        </is>
-      </c>
-      <c r="I6" s="19" t="n"/>
+          <t>Terkonfirmasi 28 Okt 2026: nominal 65.000 tetap terisi setelah ganti ke Infak (field kembali dapat diedit)</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>TC-PAY-006 (@known-bug)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="35.05" customHeight="1" s="11">
       <c r="A7" s="18" t="inlineStr">
@@ -12660,10 +12684,14 @@
       </c>
       <c r="H10" s="19" t="inlineStr">
         <is>
-          <t>Perlu verifikasi (validasi JS saat submit belum diuji)</t>
-        </is>
-      </c>
-      <c r="I10" s="19" t="n"/>
+          <t>Terkonfirmasi 28 Okt 2026: tanggal H-1 lolos constraint validation (tidak ada atribut min)</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>TC-JMP-008 (@known-bug)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="23.85" customHeight="1" s="11">
       <c r="A11" s="18" t="inlineStr">
@@ -12981,6 +13009,194 @@
         </is>
       </c>
       <c r="I17" s="19" t="n"/>
+    </row>
+    <row r="18" ht="23.85" customHeight="1" s="11">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>F-17</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Kalkulator Zakat</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>/kalkulatorzakat</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Hasil zakat perusahaan (jasa &amp; dagang/industri) dan perdagangan tidak dibulatkan. Untuk nilai yang tidak habis dibagi 40, angka desimal ikut diformat ribuan: pendapatan Rp100.000.001 menghasilkan tampilan "2.500.000.025" (terbaca 2,5 miliar).</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>Hasil dibulatkan seperti kalkulator penghasilan dan emas, mis. Rp2.500.001.</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>Fungsional / Perhitungan</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>Terkonfirmasi 28 Okt 2026 (dari script halaman, fungsi formatNumber)</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="inlineStr">
+        <is>
+          <t>Belum ada TC; usulan TC baru untuk nominal tidak bulat</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="23.85" customHeight="1" s="11">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>F-18</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Form Bayar Zakat</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>bayarzakat.baznas.go.id (tab Kalkulator)</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Kalkulator Zakat Maal memakai nisab tetap Rp82.312.725, berbeda dengan nisab per tahun Rp91.681.728 (SK Ketua BAZNAS No. 15 tahun 2026) di /kalkulatorzakat. Nisab juga dibandingkan dengan total harta sebelum dikurangi hutang.</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>Nisab konsisten dengan ketetapan terbaru dan dibandingkan dengan harta bersih sesuai ketentuan yang dikonfirmasi tim bisnis.</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>Fungsional / Konten</t>
+        </is>
+      </c>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>Terkonfirmasi dari script halaman; perlu konfirmasi tim bisnis</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>TC-PAY-020 (data uji melewati kedua nilai nisab)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="23.85" customHeight="1" s="11">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>F-19</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Kalkulator Zakat</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>/kalkulatorzakat</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Field nominal kalkulator menerima koma: input "1,5" tetap tertulis "1,5" dan dihitung sebagai 1. Minus dan karakter spesial sudah dibuang.</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>Hanya digit yang diterima.</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="inlineStr">
+        <is>
+          <t>Validasi</t>
+        </is>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>Terkonfirmasi 28 Okt 2026</t>
+        </is>
+      </c>
+      <c r="I20" s="19" t="inlineStr">
+        <is>
+          <t>TC-CALC-010 (@known-bug)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="23.85" customHeight="1" s="11">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>F-20</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Form Jemput Zakat</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>/form-jemput-zakat</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Gambar captcha tidak tampil. Endpoint gambar captcha mengembalikan pesan error PHP (fungsi pembuat gambar tidak tersedia di server), dan pesan error tersebut terlihat publik. Pengguna tidak dapat membaca kode captcha sehingga form jemput zakat tidak dapat dikirim.</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
+        <is>
+          <t>Gambar captcha tampil dan dapat di-refresh; pesan error server tidak ditampilkan ke publik.</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G21" s="19" t="inlineStr">
+        <is>
+          <t>Fungsional / Keamanan</t>
+        </is>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>Terkonfirmasi 28 Okt 2026 (konsisten pada setiap refresh)</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr">
+        <is>
+          <t>TC-JMP-003 (@known-bug)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I17"/>

</xml_diff>